<commit_message>
Learned Pivot tables and charts
</commit_message>
<xml_diff>
--- a/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
+++ b/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Documents\DSDA11\N322\AdvExcel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B6D2148-BD7D-46A1-9899-41F0E4576B77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A28BCD7C-FDC1-45AE-8F8F-251922BD4C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2590,7 +2590,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2714,10 +2714,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="21" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
@@ -2726,428 +2724,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="40">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color theme="1"/>
-        </right>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="1"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -3209,6 +2785,32 @@
         <sz val="10"/>
         <color theme="1"/>
         <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
         <scheme val="none"/>
       </font>
       <border diagonalUp="0" diagonalDown="0">
@@ -3220,6 +2822,34 @@
         <bottom/>
         <vertical/>
         <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color theme="1"/>
+        </right>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom/>
       </border>
     </dxf>
     <dxf>
@@ -3265,17 +2895,16 @@
         <sz val="10"/>
         <color theme="1"/>
         <name val="Aptos Narrow"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
         <top style="thin">
           <color theme="1"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -3319,6 +2948,32 @@
         <sz val="10"/>
         <color theme="1"/>
         <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
         <scheme val="none"/>
       </font>
       <border diagonalUp="0" diagonalDown="0">
@@ -3346,6 +3001,32 @@
         <sz val="10"/>
         <color theme="1"/>
         <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
         <scheme val="none"/>
       </font>
       <border diagonalUp="0" diagonalDown="0">
@@ -3357,6 +3038,86 @@
         <bottom/>
         <vertical/>
         <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom/>
       </border>
     </dxf>
     <dxf>
@@ -3401,6 +3162,33 @@
         <sz val="10"/>
         <color theme="1"/>
         <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
         <scheme val="none"/>
       </font>
       <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
@@ -3413,6 +3201,32 @@
         <bottom/>
         <vertical/>
         <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom/>
       </border>
     </dxf>
     <dxf>
@@ -3456,6 +3270,32 @@
         <sz val="10"/>
         <color theme="1"/>
         <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
         <scheme val="none"/>
       </font>
       <border diagonalUp="0" diagonalDown="0">
@@ -3467,6 +3307,32 @@
         <bottom/>
         <vertical/>
         <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom/>
       </border>
     </dxf>
     <dxf>
@@ -3511,6 +3377,32 @@
         <sz val="10"/>
         <color theme="1"/>
         <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
         <scheme val="none"/>
       </font>
       <border diagonalUp="0" diagonalDown="0">
@@ -3522,6 +3414,32 @@
         <bottom/>
         <vertical/>
         <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom/>
       </border>
     </dxf>
     <dxf>
@@ -3565,6 +3483,32 @@
         <sz val="11"/>
         <color theme="1"/>
         <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
         <scheme val="none"/>
       </font>
       <border diagonalUp="0" diagonalDown="0">
@@ -3592,6 +3536,32 @@
         <sz val="11"/>
         <color theme="1"/>
         <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
         <scheme val="none"/>
       </font>
       <border diagonalUp="0" diagonalDown="0">
@@ -3603,6 +3573,34 @@
         <bottom/>
         <vertical/>
         <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="1"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom/>
       </border>
     </dxf>
     <dxf>
@@ -3702,26 +3700,26 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5BA5497F-DEC0-44AB-8F20-80EF69812EB7}" name="Table2" displayName="Table2" ref="A1:P500" totalsRowCount="1" headerRowDxfId="39" dataDxfId="38" tableBorderDxfId="37">
   <autoFilter ref="A1:P499" xr:uid="{5BA5497F-DEC0-44AB-8F20-80EF69812EB7}"/>
   <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{C49FB901-6C61-48D4-8885-CD4B94CA49CC}" name="OrderID" dataDxfId="36" totalsRowDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{6F5B641F-D34D-4BF0-BD99-B4B215FD6FA9}" name="Region" dataDxfId="35" totalsRowDxfId="14"/>
-    <tableColumn id="15" xr3:uid="{E2A25365-189D-48C0-BFAF-D4926D1D02EA}" name="Updated_Region" dataDxfId="34" totalsRowDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{8377190E-9603-4D87-A476-ADEBFC3DC652}" name="Category" dataDxfId="33" totalsRowDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{A4B6F6CD-A6EE-4E43-A3F3-4CD640FCFEF0}" name="sales" totalsRowFunction="custom" dataDxfId="32" totalsRowDxfId="11">
+    <tableColumn id="1" xr3:uid="{C49FB901-6C61-48D4-8885-CD4B94CA49CC}" name="OrderID" dataDxfId="36" totalsRowDxfId="35"/>
+    <tableColumn id="2" xr3:uid="{6F5B641F-D34D-4BF0-BD99-B4B215FD6FA9}" name="Region" dataDxfId="34" totalsRowDxfId="33"/>
+    <tableColumn id="15" xr3:uid="{E2A25365-189D-48C0-BFAF-D4926D1D02EA}" name="Updated_Region" dataDxfId="32" totalsRowDxfId="31"/>
+    <tableColumn id="3" xr3:uid="{8377190E-9603-4D87-A476-ADEBFC3DC652}" name="Category" dataDxfId="30" totalsRowDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{A4B6F6CD-A6EE-4E43-A3F3-4CD640FCFEF0}" name="sales" totalsRowFunction="custom" dataDxfId="28" totalsRowDxfId="27">
       <totalsRowFormula>SUBTOTAL(9,E2:E499)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{88C8845E-E9E6-4EB3-9534-3ABD853E188F}" name="sales_category" dataDxfId="31" totalsRowDxfId="10">
+    <tableColumn id="17" xr3:uid="{88C8845E-E9E6-4EB3-9534-3ABD853E188F}" name="sales_category" dataDxfId="26" totalsRowDxfId="25">
       <calculatedColumnFormula>IF(Table2[[#This Row],[sales]]&gt;3000,"High Sales",IF(Table2[[#This Row],[sales]]&gt;1000,"Medium Sales","Low" ))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{6C72F4F4-3AA4-4C07-B02D-E31D4FA9D807}" name="discount" dataDxfId="30" totalsRowDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{EE41DADB-47D4-4FF1-9808-AE345B99EB94}" name="quantity" dataDxfId="29" totalsRowDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{C8E77239-8BEF-4765-BC91-E801E93C50FC}" name="order_date" dataDxfId="28" totalsRowDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{CE6E3ACB-BB6F-45AB-B748-BBC80F57753D}" name="delivery_date" dataDxfId="27" totalsRowDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{DB87E83D-2907-4A6E-A194-7D21A3F8D4B8}" name="customer_type" dataDxfId="26" totalsRowDxfId="5"/>
-    <tableColumn id="11" xr3:uid="{6E987BBB-89BF-49AC-B6AB-4A376A75455C}" name="payment_mode" dataDxfId="25" totalsRowDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{117FB979-FF11-4DCA-A8D6-7C90B05D3BC0}" name="profit" dataDxfId="24" totalsRowDxfId="3"/>
-    <tableColumn id="14" xr3:uid="{542039C3-2CB1-449E-B0DA-DBBF3A1CD25D}" name="Updated_City" dataDxfId="23" totalsRowDxfId="2"/>
-    <tableColumn id="13" xr3:uid="{70F2593B-A7FC-422D-BFD4-CD44CB9986C1}" name="city" dataDxfId="22" totalsRowDxfId="1"/>
-    <tableColumn id="18" xr3:uid="{A7605BF9-AA70-4D8C-B408-81E017BBE3A7}" name="Discount_Category" dataDxfId="21" totalsRowDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{6C72F4F4-3AA4-4C07-B02D-E31D4FA9D807}" name="discount" dataDxfId="24" totalsRowDxfId="23"/>
+    <tableColumn id="6" xr3:uid="{EE41DADB-47D4-4FF1-9808-AE345B99EB94}" name="quantity" dataDxfId="22" totalsRowDxfId="21"/>
+    <tableColumn id="7" xr3:uid="{C8E77239-8BEF-4765-BC91-E801E93C50FC}" name="order_date" dataDxfId="20" totalsRowDxfId="19"/>
+    <tableColumn id="8" xr3:uid="{CE6E3ACB-BB6F-45AB-B748-BBC80F57753D}" name="delivery_date" dataDxfId="18" totalsRowDxfId="17"/>
+    <tableColumn id="9" xr3:uid="{DB87E83D-2907-4A6E-A194-7D21A3F8D4B8}" name="customer_type" dataDxfId="16" totalsRowDxfId="15"/>
+    <tableColumn id="11" xr3:uid="{6E987BBB-89BF-49AC-B6AB-4A376A75455C}" name="payment_mode" dataDxfId="14" totalsRowDxfId="13"/>
+    <tableColumn id="12" xr3:uid="{117FB979-FF11-4DCA-A8D6-7C90B05D3BC0}" name="profit" dataDxfId="12" totalsRowDxfId="11"/>
+    <tableColumn id="14" xr3:uid="{542039C3-2CB1-449E-B0DA-DBBF3A1CD25D}" name="Updated_City" dataDxfId="10" totalsRowDxfId="9"/>
+    <tableColumn id="13" xr3:uid="{70F2593B-A7FC-422D-BFD4-CD44CB9986C1}" name="city" dataDxfId="8" totalsRowDxfId="7"/>
+    <tableColumn id="18" xr3:uid="{A7605BF9-AA70-4D8C-B408-81E017BBE3A7}" name="Discount_Category" dataDxfId="6" totalsRowDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6952,10 +6950,10 @@
       </c>
       <c r="P48" s="36"/>
       <c r="Q48" s="1"/>
-      <c r="R48" s="80" t="s">
+      <c r="R48" s="78" t="s">
         <v>660</v>
       </c>
-      <c r="S48" s="80" t="s">
+      <c r="S48" s="78" t="s">
         <v>594</v>
       </c>
       <c r="T48" s="1"/>
@@ -7016,7 +7014,7 @@
       </c>
       <c r="P49" s="36"/>
       <c r="Q49" s="1"/>
-      <c r="R49" s="79" t="s">
+      <c r="R49" s="77" t="s">
         <v>509</v>
       </c>
       <c r="S49" s="72">
@@ -47573,8 +47571,8 @@
   </sheetData>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="E1:F1048576">
-    <cfRule type="top10" dxfId="20" priority="3" bottom="1" rank="10"/>
-    <cfRule type="top10" dxfId="19" priority="4" rank="10"/>
+    <cfRule type="top10" dxfId="4" priority="3" bottom="1" rank="10"/>
+    <cfRule type="top10" dxfId="3" priority="4" rank="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1:G1048576">
     <cfRule type="colorScale" priority="5">
@@ -47589,7 +47587,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H1:H1048576">
-    <cfRule type="cellIs" dxfId="18" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
       <formula>5</formula>
     </cfRule>
   </conditionalFormatting>
@@ -48863,10 +48861,10 @@
   </sortState>
   <phoneticPr fontId="13" type="noConversion"/>
   <conditionalFormatting sqref="B12:B19">
-    <cfRule type="cellIs" dxfId="17" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
       <formula>65561.5</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
       <formula>50000</formula>
     </cfRule>
   </conditionalFormatting>
@@ -49294,7 +49292,7 @@
       <c r="C2" s="27">
         <v>4</v>
       </c>
-      <c r="D2" s="77">
+      <c r="D2" s="76">
         <v>46214</v>
       </c>
       <c r="E2" s="27">
@@ -49317,7 +49315,7 @@
       <c r="C3" s="27">
         <v>5</v>
       </c>
-      <c r="D3" s="77">
+      <c r="D3" s="76">
         <v>46215</v>
       </c>
       <c r="E3" s="27">
@@ -49337,7 +49335,7 @@
       <c r="C4" s="27">
         <v>3</v>
       </c>
-      <c r="D4" s="77">
+      <c r="D4" s="76">
         <v>46216</v>
       </c>
     </row>
@@ -49348,7 +49346,7 @@
       <c r="C5" s="27">
         <v>7</v>
       </c>
-      <c r="D5" s="77">
+      <c r="D5" s="76">
         <v>46217</v>
       </c>
       <c r="G5">
@@ -49363,11 +49361,10 @@
       <c r="A6" s="75">
         <v>56</v>
       </c>
-      <c r="B6" s="78" t="s">
+      <c r="B6" s="72" t="s">
         <v>710</v>
       </c>
-      <c r="C6" s="76"/>
-      <c r="D6" s="77">
+      <c r="D6" s="76">
         <v>46218</v>
       </c>
     </row>
@@ -49375,9 +49372,7 @@
       <c r="A7" s="75">
         <v>34</v>
       </c>
-      <c r="B7" s="76"/>
-      <c r="C7" s="76"/>
-      <c r="D7" s="77">
+      <c r="D7" s="76">
         <v>46219</v>
       </c>
     </row>
@@ -49385,8 +49380,7 @@
       <c r="A8" s="75">
         <v>45</v>
       </c>
-      <c r="B8" s="76"/>
-      <c r="D8" s="77">
+      <c r="D8" s="76">
         <v>46220</v>
       </c>
     </row>
@@ -49394,8 +49388,7 @@
       <c r="A9" s="75">
         <v>33</v>
       </c>
-      <c r="B9" s="76"/>
-      <c r="D9" s="77">
+      <c r="D9" s="76">
         <v>46221</v>
       </c>
     </row>
@@ -49403,8 +49396,7 @@
       <c r="A10" s="75">
         <v>45</v>
       </c>
-      <c r="B10" s="76"/>
-      <c r="D10" s="77">
+      <c r="D10" s="76">
         <v>46163</v>
       </c>
     </row>
@@ -49412,8 +49404,7 @@
       <c r="A11" s="75">
         <v>12</v>
       </c>
-      <c r="B11" s="76"/>
-      <c r="D11" s="77">
+      <c r="D11" s="76">
         <v>46164</v>
       </c>
     </row>
@@ -49421,8 +49412,7 @@
       <c r="A12" s="75">
         <v>60</v>
       </c>
-      <c r="B12" s="76"/>
-      <c r="D12" s="77">
+      <c r="D12" s="76">
         <v>46165</v>
       </c>
     </row>
@@ -49430,8 +49420,7 @@
       <c r="A13" s="75">
         <v>34</v>
       </c>
-      <c r="B13" s="76"/>
-      <c r="D13" s="77">
+      <c r="D13" s="76">
         <v>46166</v>
       </c>
     </row>
@@ -49439,7 +49428,6 @@
       <c r="A14" s="75">
         <v>68</v>
       </c>
-      <c r="B14" s="76"/>
     </row>
   </sheetData>
   <dataValidations disablePrompts="1" count="6">

</xml_diff>